<commit_message>
Implemented SauceDemo UI automation with cross-browser support
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/LoginDetails.xlsx
+++ b/src/test/resources/testdata/LoginDetails.xlsx
@@ -3,12 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30121"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F94F0968-661C-4884-84C0-C4EA976DDB22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5AD1606A-3275-4C8F-B019-35F9C6FB8784}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="LoginData" sheetId="1" r:id="rId1"/>
+    <sheet name="ValidLogin" sheetId="1" r:id="rId1"/>
+    <sheet name="InvalidLogin" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -31,6 +32,44 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="11">
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>secret_sauce</t>
+  </si>
+  <si>
+    <t>expectedMessage</t>
+  </si>
+  <si>
+    <t>locked_out_user</t>
+  </si>
+  <si>
+    <t>Epic sadface</t>
+  </si>
+  <si>
+    <t>invalid_user</t>
+  </si>
+  <si>
+    <t>wrongpass</t>
+  </si>
+  <si>
+    <t>Username is required</t>
+  </si>
+  <si>
+    <t>Password is required</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -380,9 +419,95 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC424D96-D941-4A76-AC05-8F1F4028FA17}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>